<commit_message>
fixed issues from merging
</commit_message>
<xml_diff>
--- a/env/TestData.xlsx
+++ b/env/TestData.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <workbookPr codeName="ThisWorkbook"/>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Sheet" sheetId="1" r:id="rId1"/>
   </sheets>
 </workbook>
 </file>
@@ -32,11 +32,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:vt="http://schemas.openxmlformats.org/officeDocument/2006/docPropsVTypes">
-  <numFmts count="4">
+  <numFmts count="3">
     <numFmt numFmtId="56" formatCode="&quot;上午/下午 &quot;hh&quot;時&quot;mm&quot;分&quot;ss&quot;秒 &quot;"/>
-    <numFmt numFmtId="164" formatCode="[$-F800]dddd\,\ mmmm\ dd\,\ yyyy"/>
-    <numFmt numFmtId="165" formatCode="yyyy-mm-dd h:mm:ss"/>
-    <numFmt numFmtId="166" formatCode="YYYY-MM-DD HH:MM"/>
+    <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
+    <numFmt numFmtId="165" formatCode="YYYY-MM-DD HH:MM"/>
   </numFmts>
   <fonts count="1">
     <font>
@@ -400,7 +399,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E41"/>
+  <dimension ref="A1:E30"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -427,10 +426,10 @@
         <v>Alice Green</v>
       </c>
       <c r="C2" t="str">
-        <v>Thursday, March 12, 2026</v>
+        <v>2026-02-03 09:00</v>
       </c>
       <c r="D2" t="str">
-        <v>45.00</v>
+        <v>45</v>
       </c>
       <c r="E2" t="str">
         <v>U001</v>
@@ -438,67 +437,220 @@
     </row>
     <row r="3">
       <c r="A3" t="str">
+        <v>P004</v>
+      </c>
+      <c r="B3" t="str">
+        <v>David Brown</v>
+      </c>
+      <c r="C3" t="str">
+        <v>2026-02-03 11:00</v>
+      </c>
+      <c r="D3" t="str">
+        <v>60</v>
+      </c>
+      <c r="E3" t="str">
+        <v>U002</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>P007</v>
+      </c>
+      <c r="B4" t="str">
+        <v>Grace Taylor</v>
+      </c>
+      <c r="C4" t="str">
+        <v>2026-02-10 14:30</v>
+      </c>
+      <c r="D4" t="str">
+        <v>30</v>
+      </c>
+      <c r="E4" t="str">
+        <v>U001</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
         <v>P002</v>
       </c>
-      <c r="B3" t="str">
+      <c r="B5" t="str">
         <v>Bob Smith</v>
       </c>
-      <c r="C3" t="str">
-        <v>Wednesday, March 11, 2026</v>
-      </c>
-      <c r="D3" t="str">
-        <v>60.00</v>
-      </c>
-      <c r="E3" t="str">
-        <v>U002</v>
+      <c r="C5" t="str">
+        <v>2026-02-17 09:00</v>
+      </c>
+      <c r="D5" t="str">
+        <v>60</v>
+      </c>
+      <c r="E5" t="str">
+        <v>U002</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>P005</v>
+      </c>
+      <c r="B6" t="str">
+        <v>Emma Wilson</v>
+      </c>
+      <c r="C6" t="str">
+        <v>2026-02-17 11:00</v>
+      </c>
+      <c r="D6" t="str">
+        <v>45</v>
+      </c>
+      <c r="E6" t="str">
+        <v>U001</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>P008</v>
+      </c>
+      <c r="B7" t="str">
+        <v>Hannah Lewis</v>
+      </c>
+      <c r="C7" t="str">
+        <v>2026-02-17 14:00</v>
+      </c>
+      <c r="D7" t="str">
+        <v>30</v>
+      </c>
+      <c r="E7" t="str">
+        <v>U002</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>P003</v>
+      </c>
+      <c r="B8" t="str">
+        <v>Carol White</v>
+      </c>
+      <c r="C8" t="str">
+        <v>2026-02-24 09:30</v>
+      </c>
+      <c r="D8" t="str">
+        <v>60</v>
+      </c>
+      <c r="E8" t="str">
+        <v>U001</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>P006</v>
+      </c>
+      <c r="B9" t="str">
+        <v>Frank Moore</v>
+      </c>
+      <c r="C9" t="str">
+        <v>2026-03-04 10:30</v>
+      </c>
+      <c r="D9" t="str">
+        <v>120</v>
+      </c>
+      <c r="E9" t="str">
+        <v>U002</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>P010</v>
+      </c>
+      <c r="B10" t="str">
+        <v>Julia Thompson</v>
+      </c>
+      <c r="C10" t="str">
+        <v>2026-03-05 14:21</v>
+      </c>
+      <c r="D10" t="str">
+        <v>60</v>
+      </c>
+      <c r="E10" t="str">
+        <v>U001</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v>P002</v>
+      </c>
+      <c r="B11" t="str">
+        <v>Bob Smith</v>
+      </c>
+      <c r="C11" t="str">
+        <v>2026-03-06 14:00</v>
+      </c>
+      <c r="D11" t="str">
+        <v>60</v>
+      </c>
+      <c r="E11" t="str">
+        <v>U002</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v>P009</v>
+      </c>
+      <c r="B12" t="str">
+        <v>Ivan Martin</v>
+      </c>
+      <c r="C12" t="str">
+        <v>2026-03-09 08:30</v>
+      </c>
+      <c r="D12" t="str">
+        <v>45</v>
+      </c>
+      <c r="E12" t="str">
+        <v>U001</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>P003</v>
+        <v>P004</v>
       </c>
       <c r="B13" t="str">
-        <v>Alice Green</v>
+        <v>David Brown</v>
       </c>
       <c r="C13" t="str">
-        <v>2026-02-03 09:00</v>
+        <v>2026-03-11 09:00</v>
       </c>
       <c r="D13" t="str">
-        <v>45</v>
+        <v>30</v>
       </c>
       <c r="E13" t="str">
-        <v>U001</v>
+        <v>U002</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>P004</v>
+        <v>P007</v>
       </c>
       <c r="B14" t="str">
-        <v>James Carter</v>
+        <v>Grace Taylor</v>
       </c>
       <c r="C14" t="str">
-        <v>2026-02-03 11:00</v>
+        <v>2026-03-11 14:00</v>
       </c>
       <c r="D14" t="str">
         <v>60</v>
       </c>
       <c r="E14" t="str">
-        <v>U003</v>
+        <v>U001</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>P005</v>
+        <v>P001</v>
       </c>
       <c r="B15" t="str">
-        <v>Carol White</v>
+        <v>Alice Green</v>
       </c>
       <c r="C15" t="str">
-        <v>2026-02-10 14:30</v>
+        <v>2026-03-16 10:00</v>
       </c>
       <c r="D15" t="str">
-        <v>30</v>
+        <v>90</v>
       </c>
       <c r="E15" t="str">
         <v>U002</v>
@@ -506,16 +658,16 @@
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>P006</v>
+        <v>P005</v>
       </c>
       <c r="B16" t="str">
-        <v>David Brown</v>
+        <v>Emma Wilson</v>
       </c>
       <c r="C16" t="str">
-        <v>2026-02-17 09:00</v>
+        <v>2026-03-18 09:00</v>
       </c>
       <c r="D16" t="str">
-        <v>60</v>
+        <v>45</v>
       </c>
       <c r="E16" t="str">
         <v>U001</v>
@@ -523,19 +675,19 @@
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>P007</v>
+        <v>P003</v>
       </c>
       <c r="B17" t="str">
-        <v>Emma Wilson</v>
+        <v>Carol White</v>
       </c>
       <c r="C17" t="str">
-        <v>2026-02-17 11:00</v>
+        <v>2026-03-18 14:00</v>
       </c>
       <c r="D17" t="str">
-        <v>45</v>
+        <v>60</v>
       </c>
       <c r="E17" t="str">
-        <v>U004</v>
+        <v>U002</v>
       </c>
     </row>
     <row r="18">
@@ -543,33 +695,33 @@
         <v>P008</v>
       </c>
       <c r="B18" t="str">
-        <v>Frank Moore</v>
+        <v>Hannah Lewis</v>
       </c>
       <c r="C18" t="str">
-        <v>2026-02-17 14:00</v>
+        <v>2026-03-23 09:00</v>
       </c>
       <c r="D18" t="str">
         <v>30</v>
       </c>
       <c r="E18" t="str">
-        <v>U002</v>
+        <v>U001</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>P009</v>
+        <v>P006</v>
       </c>
       <c r="B19" t="str">
-        <v>Grace Taylor</v>
+        <v>Frank Moore</v>
       </c>
       <c r="C19" t="str">
-        <v>2026-02-24 09:30</v>
+        <v>2026-03-25 09:00</v>
       </c>
       <c r="D19" t="str">
-        <v>60</v>
+        <v>45</v>
       </c>
       <c r="E19" t="str">
-        <v>U003</v>
+        <v>U002</v>
       </c>
     </row>
     <row r="20">
@@ -577,13 +729,13 @@
         <v>P010</v>
       </c>
       <c r="B20" t="str">
-        <v>Steve Adams</v>
+        <v>Julia Thompson</v>
       </c>
       <c r="C20" t="str">
-        <v>2026-03-04 10:30</v>
+        <v>2026-03-25 11:00</v>
       </c>
       <c r="D20" t="str">
-        <v>120</v>
+        <v>45</v>
       </c>
       <c r="E20" t="str">
         <v>U001</v>
@@ -591,13 +743,13 @@
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>P011</v>
+        <v>P002</v>
       </c>
       <c r="B21" t="str">
-        <v>Barry Jones</v>
+        <v>Bob Smith</v>
       </c>
       <c r="C21" t="str">
-        <v>2026-03-05 14:21</v>
+        <v>2026-03-25 14:00</v>
       </c>
       <c r="D21" t="str">
         <v>60</v>
@@ -608,64 +760,64 @@
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>P012</v>
+        <v>P004</v>
       </c>
       <c r="B22" t="str">
-        <v>Bob Harris</v>
+        <v>David Brown</v>
       </c>
       <c r="C22" t="str">
-        <v>2026-03-06 14:00</v>
+        <v>2026-03-30 10:00</v>
       </c>
       <c r="D22" t="str">
-        <v>60</v>
+        <v>90</v>
       </c>
       <c r="E22" t="str">
-        <v>U004</v>
+        <v>U001</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>P013</v>
+        <v>P009</v>
       </c>
       <c r="B23" t="str">
-        <v>Hannah Lewis</v>
+        <v>Ivan Martin</v>
       </c>
       <c r="C23" t="str">
-        <v>2026-03-09 08:30</v>
+        <v>2026-04-01 09:00</v>
       </c>
       <c r="D23" t="str">
         <v>45</v>
       </c>
       <c r="E23" t="str">
-        <v>U001</v>
+        <v>U002</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>P014</v>
+        <v>P001</v>
       </c>
       <c r="B24" t="str">
-        <v>Ivan Martin</v>
+        <v>Alice Green</v>
       </c>
       <c r="C24" t="str">
-        <v>2026-03-11 09:00</v>
+        <v>2026-04-01 11:00</v>
       </c>
       <c r="D24" t="str">
-        <v>30</v>
+        <v>45</v>
       </c>
       <c r="E24" t="str">
-        <v>U003</v>
+        <v>U001</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>P015</v>
+        <v>P007</v>
       </c>
       <c r="B25" t="str">
-        <v>Julia Thompson</v>
+        <v>Grace Taylor</v>
       </c>
       <c r="C25" t="str">
-        <v>2026-03-11 14:00</v>
+        <v>2026-04-07 14:00</v>
       </c>
       <c r="D25" t="str">
         <v>60</v>
@@ -676,16 +828,16 @@
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>P016</v>
+        <v>P003</v>
       </c>
       <c r="B26" t="str">
-        <v>Kevin Garcia</v>
+        <v>Carol White</v>
       </c>
       <c r="C26" t="str">
-        <v>2026-03-16 10:00</v>
+        <v>2026-04-14 09:00</v>
       </c>
       <c r="D26" t="str">
-        <v>90</v>
+        <v>30</v>
       </c>
       <c r="E26" t="str">
         <v>U001</v>
@@ -693,50 +845,50 @@
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>P017</v>
+        <v>P008</v>
       </c>
       <c r="B27" t="str">
-        <v>Laura Martinez</v>
+        <v>Hannah Lewis</v>
       </c>
       <c r="C27" t="str">
-        <v>2026-03-18 09:00</v>
+        <v>2026-04-14 13:00</v>
       </c>
       <c r="D27" t="str">
-        <v>45</v>
+        <v>60</v>
       </c>
       <c r="E27" t="str">
-        <v>U004</v>
+        <v>U002</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v>P018</v>
+        <v>P005</v>
       </c>
       <c r="B28" t="str">
-        <v>Marcus Robinson</v>
+        <v>Emma Wilson</v>
       </c>
       <c r="C28" t="str">
-        <v>2026-03-18 14:00</v>
+        <v>2026-04-20 09:30</v>
       </c>
       <c r="D28" t="str">
-        <v>60</v>
+        <v>90</v>
       </c>
       <c r="E28" t="str">
-        <v>U003</v>
+        <v>U001</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v>P019</v>
+        <v>P010</v>
       </c>
       <c r="B29" t="str">
-        <v>Nina Clark</v>
+        <v>Julia Thompson</v>
       </c>
       <c r="C29" t="str">
-        <v>2026-03-23 09:00</v>
+        <v>2026-04-22 13:00</v>
       </c>
       <c r="D29" t="str">
-        <v>30</v>
+        <v>45</v>
       </c>
       <c r="E29" t="str">
         <v>U002</v>
@@ -744,211 +896,24 @@
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v>P020</v>
+        <v>P006</v>
       </c>
       <c r="B30" t="str">
-        <v>Oliver Rodriguez</v>
+        <v>Frank Moore</v>
       </c>
       <c r="C30" t="str">
-        <v>2026-03-25 09:00</v>
+        <v>2026-04-28 15:00</v>
       </c>
       <c r="D30" t="str">
-        <v>45</v>
+        <v>60</v>
       </c>
       <c r="E30" t="str">
-        <v>U001</v>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" t="str">
-        <v>P021</v>
-      </c>
-      <c r="B31" t="str">
-        <v>Paula Lewis</v>
-      </c>
-      <c r="C31" t="str">
-        <v>2026-03-25 11:00</v>
-      </c>
-      <c r="D31" t="str">
-        <v>45</v>
-      </c>
-      <c r="E31" t="str">
-        <v>U004</v>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" t="str">
-        <v>P022</v>
-      </c>
-      <c r="B32" t="str">
-        <v>Quinn Walker</v>
-      </c>
-      <c r="C32" t="str">
-        <v>2026-03-25 14:00</v>
-      </c>
-      <c r="D32" t="str">
-        <v>60</v>
-      </c>
-      <c r="E32" t="str">
-        <v>U002</v>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" t="str">
-        <v>P023</v>
-      </c>
-      <c r="B33" t="str">
-        <v>Rachel Hall</v>
-      </c>
-      <c r="C33" t="str">
-        <v>2026-03-30 10:00</v>
-      </c>
-      <c r="D33" t="str">
-        <v>90</v>
-      </c>
-      <c r="E33" t="str">
-        <v>U003</v>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" t="str">
-        <v>P024</v>
-      </c>
-      <c r="B34" t="str">
-        <v>Sam Allen</v>
-      </c>
-      <c r="C34" t="str">
-        <v>2026-04-01 09:00</v>
-      </c>
-      <c r="D34" t="str">
-        <v>45</v>
-      </c>
-      <c r="E34" t="str">
-        <v>U001</v>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" t="str">
-        <v>P025</v>
-      </c>
-      <c r="B35" t="str">
-        <v>Tina Young</v>
-      </c>
-      <c r="C35" t="str">
-        <v>2026-04-01 11:00</v>
-      </c>
-      <c r="D35" t="str">
-        <v>45</v>
-      </c>
-      <c r="E35" t="str">
-        <v>U002</v>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" t="str">
-        <v>P026</v>
-      </c>
-      <c r="B36" t="str">
-        <v>Uma Hernandez</v>
-      </c>
-      <c r="C36" t="str">
-        <v>2026-04-07 14:00</v>
-      </c>
-      <c r="D36" t="str">
-        <v>60</v>
-      </c>
-      <c r="E36" t="str">
-        <v>U004</v>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" t="str">
-        <v>P027</v>
-      </c>
-      <c r="B37" t="str">
-        <v>Victor King</v>
-      </c>
-      <c r="C37" t="str">
-        <v>2026-04-14 09:00</v>
-      </c>
-      <c r="D37" t="str">
-        <v>30</v>
-      </c>
-      <c r="E37" t="str">
-        <v>U001</v>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" t="str">
-        <v>P028</v>
-      </c>
-      <c r="B38" t="str">
-        <v>Wendy Wright</v>
-      </c>
-      <c r="C38" t="str">
-        <v>2026-04-14 13:00</v>
-      </c>
-      <c r="D38" t="str">
-        <v>60</v>
-      </c>
-      <c r="E38" t="str">
-        <v>U003</v>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" t="str">
-        <v>P029</v>
-      </c>
-      <c r="B39" t="str">
-        <v>Xander Scott</v>
-      </c>
-      <c r="C39" t="str">
-        <v>2026-04-20 09:30</v>
-      </c>
-      <c r="D39" t="str">
-        <v>90</v>
-      </c>
-      <c r="E39" t="str">
-        <v>U002</v>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" t="str">
-        <v>P030</v>
-      </c>
-      <c r="B40" t="str">
-        <v>Yasmin Green</v>
-      </c>
-      <c r="C40" t="str">
-        <v>2026-04-22 13:00</v>
-      </c>
-      <c r="D40" t="str">
-        <v>45</v>
-      </c>
-      <c r="E40" t="str">
-        <v>U004</v>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" t="str">
-        <v>P031</v>
-      </c>
-      <c r="B41" t="str">
-        <v>Zoe Baker</v>
-      </c>
-      <c r="C41" t="str">
-        <v>2026-04-28 15:00</v>
-      </c>
-      <c r="D41" t="str">
-        <v>60</v>
-      </c>
-      <c r="E41" t="str">
         <v>U001</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E41"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E30"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>